<commit_message>
investment add and generating balances fun create
</commit_message>
<xml_diff>
--- a/balance_generate/dictionaries/amort_type.xlsx
+++ b/balance_generate/dictionaries/amort_type.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD904641-8274-4F6D-B2AD-6ABE6864BD05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE6BD05-B44D-466A-AD59-712781FF3715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6400" yWindow="1820" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>bullet</t>
   </si>
@@ -34,6 +34,9 @@
   </si>
   <si>
     <t>constant_amort</t>
+  </si>
+  <si>
+    <t>non_standard</t>
   </si>
 </sst>
 </file>
@@ -351,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.08984375" customWidth="1"/>
@@ -381,6 +384,14 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>